<commit_message>
Add Sample Feedback Google Form link and update default template format with Ramco Institute & B.Tech IT
</commit_message>
<xml_diff>
--- a/frontend/public/sample_recipient_template.xlsx
+++ b/frontend/public/sample_recipient_template.xlsx
@@ -401,19 +401,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Name(Eg: Kirran S T - IV IT)</v>
+        <v>Name (Eg: Kirran S T)</v>
       </c>
       <c r="B1" t="str">
-        <v>Email(Eg: test@gmail.com)</v>
+        <v>Email (Eg: kirranvijay@gmail.com)</v>
       </c>
       <c r="C1" t="str">
-        <v>Department(Eg: IT)</v>
+        <v>Department (Eg: B.Tech IT)</v>
       </c>
       <c r="D1" t="str">
-        <v>College(Eg: St. Joseph's)</v>
+        <v>Year (Eg: IV Year)</v>
       </c>
       <c r="E1" t="str">
-        <v>Year(Eg: IV Year)</v>
+        <v>College (Eg: Ramco Institute Of Technology)</v>
       </c>
       <c r="F1" t="str">
         <v>How was the event? (Feedback / Remarks)</v>
@@ -430,13 +430,13 @@
         <v>kirranvijay@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>Information Technology</v>
+        <v>B.Tech IT</v>
       </c>
       <c r="D2" t="str">
-        <v>St. Joseph's College of Engineering</v>
+        <v>IV Year</v>
       </c>
       <c r="E2" t="str">
-        <v>IV Year</v>
+        <v>Ramco Institute Of Technology</v>
       </c>
       <c r="F2" t="str">
         <v>Excellent workshop and very well organized!</v>
@@ -453,13 +453,13 @@
         <v>kirranvijay@gmail.com</v>
       </c>
       <c r="C3" t="str">
-        <v>IT</v>
+        <v>Information Technology</v>
       </c>
       <c r="D3" t="str">
-        <v>St. Joseph's College of Engineering</v>
+        <v>4th Year</v>
       </c>
       <c r="E3" t="str">
-        <v>4th Year</v>
+        <v>Ramco Institute Of Technology</v>
       </c>
       <c r="F3" t="str">
         <v>Great hands-on learning experience.</v>

</xml_diff>